<commit_message>
Radars inline dans chaque section + scoring Excel avec radars + lien download dans sidebar
</commit_message>
<xml_diff>
--- a/benchmark-cartier.xlsx
+++ b/benchmark-cartier.xlsx
@@ -8,12 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="Réponses complètes" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Grille de scoring" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Méthodologie" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Scoring &amp; Radars" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Grille de scoring" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Méthodologie" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Réponses complètes'!$A$1:$K$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Grille de scoring'!$A$1:$K$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Grille de scoring'!$A$1:$K$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,6 +50,12 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00B8965A"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="6">
@@ -109,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -133,6 +140,20 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -209,7 +230,936 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Découverte</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <radarChart>
+        <radarStyle val="filled"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>GPT-4o</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Scoring &amp; Radars'!$B$5:$F$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>Perplexity</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Scoring &amp; Radars'!$B$6:$F$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <v>Claude</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Scoring &amp; Radars'!$B$7:$F$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </radarChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Comparaison</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <radarChart>
+        <radarStyle val="filled"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>GPT-4o</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Scoring &amp; Radars'!$B$12:$F$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>Perplexity</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Scoring &amp; Radars'!$B$13:$F$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <v>Claude</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Scoring &amp; Radars'!$B$14:$F$14</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </radarChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Validation</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <radarChart>
+        <radarStyle val="filled"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>GPT-4o</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Scoring &amp; Radars'!$B$19:$F$19</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>Perplexity</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Scoring &amp; Radars'!$B$20:$F$20</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <v>Claude</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Scoring &amp; Radars'!$B$21:$F$21</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </radarChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Parcours</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <radarChart>
+        <radarStyle val="filled"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>GPT-4o</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Scoring &amp; Radars'!$B$26:$F$26</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>Perplexity</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Scoring &amp; Radars'!$B$27:$F$27</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <v>Claude</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Scoring &amp; Radars'!$B$28:$F$28</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </radarChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Investissement</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <radarChart>
+        <radarStyle val="filled"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>GPT-4o</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Scoring &amp; Radars'!$B$33:$F$33</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>Perplexity</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Scoring &amp; Radars'!$B$34:$F$34</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <v>Claude</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Scoring &amp; Radars'!$B$35:$F$35</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </radarChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Substitution</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <radarChart>
+        <radarStyle val="filled"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>GPT-4o</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Scoring &amp; Radars'!$B$40:$F$40</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>Perplexity</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Scoring &amp; Radars'!$B$41:$F$41</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <v>Claude</v>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Scoring &amp; Radars'!$B$42:$F$42</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </radarChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>31</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="5" name="Chart 5"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>38</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="6" name="Chart 6"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId6"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -232,6 +1182,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1862,6 +2815,751 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Scoring par catégorie — Benchmark Cartier</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>Découverte</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Plateforme</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Présence</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>Exactitude</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>Narratif</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>Actionnabilité</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>Total /25</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>GPT-4o</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C5" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" s="15" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G5" s="16" t="n">
+        <v>18.7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Perplexity</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="C6" s="15" t="n">
+        <v>2.67</v>
+      </c>
+      <c r="D6" s="15" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="E6" s="15" t="n">
+        <v>2.67</v>
+      </c>
+      <c r="F6" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="16" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="16" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>Comparaison</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Plateforme</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Présence</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Exactitude</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>Narratif</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>Actionnabilité</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="inlineStr">
+        <is>
+          <t>Total /25</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>GPT-4o</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" s="15" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="D12" s="15" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="E12" s="15" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="F12" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="G12" s="16" t="n">
+        <v>19.7</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Perplexity</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="C13" s="15" t="n">
+        <v>2.67</v>
+      </c>
+      <c r="D13" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E13" s="15" t="n">
+        <v>2.67</v>
+      </c>
+      <c r="F13" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="G13" s="16" t="n">
+        <v>15.7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C14" s="15" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="D14" s="15" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="E14" s="15" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="F14" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="G14" s="16" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Plateforme</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Présence</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Exactitude</t>
+        </is>
+      </c>
+      <c r="E18" s="13" t="inlineStr">
+        <is>
+          <t>Narratif</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>Actionnabilité</t>
+        </is>
+      </c>
+      <c r="G18" s="13" t="inlineStr">
+        <is>
+          <t>Total /25</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>GPT-4o</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C19" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D19" s="15" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="E19" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F19" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G19" s="16" t="n">
+        <v>19.7</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>Perplexity</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C20" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D20" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E20" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F20" s="15" t="n">
+        <v>2.67</v>
+      </c>
+      <c r="G20" s="16" t="n">
+        <v>19.7</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C21" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21" s="15" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="E21" s="15" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="F21" s="15" t="n">
+        <v>2.67</v>
+      </c>
+      <c r="G21" s="16" t="n">
+        <v>19.7</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>Parcours</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>Plateforme</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>Présence</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>Exactitude</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>Narratif</t>
+        </is>
+      </c>
+      <c r="F25" s="13" t="inlineStr">
+        <is>
+          <t>Actionnabilité</t>
+        </is>
+      </c>
+      <c r="G25" s="13" t="inlineStr">
+        <is>
+          <t>Total /25</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>GPT-4o</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C26" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D26" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E26" s="15" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="F26" s="15" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="G26" s="16" t="n">
+        <v>21.3</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>Perplexity</t>
+        </is>
+      </c>
+      <c r="B27" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C27" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D27" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E27" s="15" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="F27" s="15" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="G27" s="16" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C28" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D28" s="15" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="E28" s="15" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="F28" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="G28" s="16" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>Investissement</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>Plateforme</t>
+        </is>
+      </c>
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>Présence</t>
+        </is>
+      </c>
+      <c r="C32" s="13" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="inlineStr">
+        <is>
+          <t>Exactitude</t>
+        </is>
+      </c>
+      <c r="E32" s="13" t="inlineStr">
+        <is>
+          <t>Narratif</t>
+        </is>
+      </c>
+      <c r="F32" s="13" t="inlineStr">
+        <is>
+          <t>Actionnabilité</t>
+        </is>
+      </c>
+      <c r="G32" s="13" t="inlineStr">
+        <is>
+          <t>Total /25</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t>GPT-4o</t>
+        </is>
+      </c>
+      <c r="B33" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C33" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D33" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E33" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="F33" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G33" s="16" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>Perplexity</t>
+        </is>
+      </c>
+      <c r="B34" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C34" s="15" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="D34" s="15" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="E34" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F34" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G34" s="16" t="n">
+        <v>17.7</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="18" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="B35" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C35" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D35" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E35" s="15" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="F35" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G35" s="16" t="n">
+        <v>18.7</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>Substitution</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>Plateforme</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>Présence</t>
+        </is>
+      </c>
+      <c r="C39" s="13" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="D39" s="13" t="inlineStr">
+        <is>
+          <t>Exactitude</t>
+        </is>
+      </c>
+      <c r="E39" s="13" t="inlineStr">
+        <is>
+          <t>Narratif</t>
+        </is>
+      </c>
+      <c r="F39" s="13" t="inlineStr">
+        <is>
+          <t>Actionnabilité</t>
+        </is>
+      </c>
+      <c r="G39" s="13" t="inlineStr">
+        <is>
+          <t>Total /25</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>GPT-4o</t>
+        </is>
+      </c>
+      <c r="B40" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C40" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D40" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E40" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="F40" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G40" s="16" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="17" t="inlineStr">
+        <is>
+          <t>Perplexity</t>
+        </is>
+      </c>
+      <c r="B41" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C41" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D41" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E41" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="F41" s="15" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G41" s="16" t="n">
+        <v>18.5</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="18" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="B42" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C42" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D42" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E42" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F42" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="G42" s="16" t="n">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3369,7 +5067,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3388,7 +5086,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
@@ -3417,7 +5114,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -3439,7 +5135,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>

</xml_diff>